<commit_message>
Updated checks to include thermal relief constraints
</commit_message>
<xml_diff>
--- a/hardware/pcb-checklist.xlsx
+++ b/hardware/pcb-checklist.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="45">
   <si>
     <t xml:space="preserve">Item</t>
   </si>
@@ -52,10 +52,13 @@
     <t xml:space="preserve">Mark diode direction - not using default footprint (hard to identify)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hide order number</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Text in hidden area, type JLC four times so JLCJLCJLCJLC</t>
+    <t xml:space="preserve">Set fill zone thermal relief</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.3mm gap, 0.4mm spoke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F.Cu,B.Cu</t>
   </si>
   <si>
     <t xml:space="preserve">Tooling holes (Fiducials)</t>
@@ -513,7 +516,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.57"/>
@@ -573,26 +576,26 @@
         <v>11</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>5</v>
@@ -600,10 +603,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>5</v>
@@ -611,10 +614,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>18</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>5</v>
@@ -622,10 +625,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>5</v>
@@ -633,106 +636,107 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
         <v>40</v>
       </c>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="1" t="s">
+      <c r="A23" s="2" t="s">
         <v>41</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A21:C21"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A20" r:id="rId1" display="https://jlcpcb.com/help/article/how-to-generate-gerber-and-drill-files-in-kicad-7"/>
+    <hyperlink ref="A21" r:id="rId1" display="https://jlcpcb.com/help/article/how-to-generate-gerber-and-drill-files-in-kicad-7"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>